<commit_message>
Short runs finished for all power tests
</commit_message>
<xml_diff>
--- a/results/power/power_results_by_hierarchy.xlsx
+++ b/results/power/power_results_by_hierarchy.xlsx
@@ -8,14 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\riscv-power-aware\results\power\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{464105DF-2152-43BC-9BF0-8A3D267133B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07192F74-FEE2-423D-9EC3-5353FABDE7A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{71665766-232F-42B5-8C54-1F711CA08D87}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{71665766-232F-42B5-8C54-1F711CA08D87}"/>
   </bookViews>
   <sheets>
     <sheet name="power_spin" sheetId="1" r:id="rId1"/>
     <sheet name="power_alu" sheetId="2" r:id="rId2"/>
     <sheet name="power_mem" sheetId="3" r:id="rId3"/>
+    <sheet name="power_branch" sheetId="4" r:id="rId4"/>
+    <sheet name="power_chase" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="681" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1135" uniqueCount="192">
   <si>
     <t>Global Resources</t>
   </si>
@@ -707,7 +709,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="9">
     <dxf>
       <font>
         <b/>
@@ -745,6 +747,82 @@
           <color theme="4" tint="0.39997558519241921"/>
         </top>
       </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -788,7 +866,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{B15E26C1-E4F4-4784-804C-75044EEC47E0}" name="Table3" displayName="Table3" ref="A1:E76" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="1" tableBorderDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{B15E26C1-E4F4-4784-804C-75044EEC47E0}" name="Table3" displayName="Table3" ref="A1:E76" totalsRowShown="0" headerRowDxfId="8" headerRowBorderDxfId="7" tableBorderDxfId="6">
   <autoFilter ref="A1:E76" xr:uid="{B15E26C1-E4F4-4784-804C-75044EEC47E0}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E76">
     <sortCondition descending="1" ref="B1:B76"/>
@@ -799,6 +877,34 @@
     <tableColumn id="3" xr3:uid="{B363E05E-A591-4722-825D-DF06189F9DF4}" name="Current Level Dynamic On-Chip Power (W)"/>
     <tableColumn id="4" xr3:uid="{E3DFC169-377F-4E92-96BF-7E85B405F942}" name="Full Hierarchy Name"/>
     <tableColumn id="5" xr3:uid="{4BFBB5ED-CF9F-4289-B2D1-A5DE474D6F53}" name="Entity Name"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{6621A618-A607-45B2-8D2F-D68FB4900DC2}" name="Table4" displayName="Table4" ref="A1:E76" totalsRowShown="0" headerRowDxfId="3" headerRowBorderDxfId="4" tableBorderDxfId="5">
+  <autoFilter ref="A1:E76" xr:uid="{6621A618-A607-45B2-8D2F-D68FB4900DC2}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{45346CE6-87DC-4E53-9D5D-79D6CDEE6798}" name="Compilation Hierarchy Node"/>
+    <tableColumn id="2" xr3:uid="{92B9C947-037A-4AB7-8BCD-F0AEA50A1929}" name="Cumulative Dynamic On-Chip Power (W)"/>
+    <tableColumn id="3" xr3:uid="{AE20CBAF-A324-4755-A507-3DC2671D9516}" name="Current Level Dynamic On-Chip Power (W)"/>
+    <tableColumn id="4" xr3:uid="{371800DC-067A-4BAA-99FE-A6D1B76213D3}" name="Full Hierarchy Name"/>
+    <tableColumn id="5" xr3:uid="{DC92EB74-D179-4636-BC18-236265F0F357}" name="Entity Name"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{661AF9EA-031A-48DC-B7AF-72B2D6F955FE}" name="Table5" displayName="Table5" ref="A1:E76" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="1" tableBorderDxfId="2">
+  <autoFilter ref="A1:E76" xr:uid="{661AF9EA-031A-48DC-B7AF-72B2D6F955FE}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{FAFD6D57-E89E-434D-A461-63F04DC7AA96}" name="Compilation Hierarchy Node"/>
+    <tableColumn id="2" xr3:uid="{8B454DF6-1269-4CC1-BCD9-D845C7509202}" name="Cumulative Dynamic On-Chip Power (W)"/>
+    <tableColumn id="3" xr3:uid="{49CBF02C-88E6-49ED-9800-97DE0CCC66EC}" name="Current Level Dynamic On-Chip Power (W)"/>
+    <tableColumn id="4" xr3:uid="{68F0631B-A17A-4CCA-8F48-28DF685777A9}" name="Full Hierarchy Name"/>
+    <tableColumn id="5" xr3:uid="{1C5F9945-1865-4A8A-9FEB-E9D09FE1B421}" name="Entity Name"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5026,4 +5132,2610 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9342C08-D979-4FBE-81C9-BC1102F1F095}">
+  <dimension ref="A1:E76"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="28.7109375" customWidth="1"/>
+    <col min="2" max="2" width="39.5703125" customWidth="1"/>
+    <col min="3" max="3" width="41.42578125" customWidth="1"/>
+    <col min="4" max="4" width="85.7109375" customWidth="1"/>
+    <col min="5" max="5" width="57.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>0.33500000000000002</v>
+      </c>
+      <c r="C2">
+        <v>0.27200000000000002</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>6.4000000000000001E-2</v>
+      </c>
+      <c r="C3">
+        <v>1.0999999999999999E-2</v>
+      </c>
+      <c r="E3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>4.5999999999999999E-2</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5">
+        <v>4.5999999999999999E-2</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>4.5999999999999999E-2</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7">
+        <v>4.5999999999999999E-2</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8">
+        <v>4.5999999999999999E-2</v>
+      </c>
+      <c r="C8">
+        <v>4.5999999999999999E-2</v>
+      </c>
+      <c r="D8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9">
+        <v>6.0000000000000001E-3</v>
+      </c>
+      <c r="C9" s="1">
+        <v>6.9700000000000003E-4</v>
+      </c>
+      <c r="D9" t="s">
+        <v>18</v>
+      </c>
+      <c r="E9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10">
+        <v>1E-3</v>
+      </c>
+      <c r="C10" s="1">
+        <v>6.7900000000000002E-6</v>
+      </c>
+      <c r="D10" t="s">
+        <v>21</v>
+      </c>
+      <c r="E10" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" s="1">
+        <v>8.7699999999999996E-4</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="1">
+        <v>8.7699999999999996E-4</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13" s="1">
+        <v>8.7699999999999996E-4</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
+      </c>
+      <c r="D13" t="s">
+        <v>30</v>
+      </c>
+      <c r="E13" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" s="1">
+        <v>8.7699999999999996E-4</v>
+      </c>
+      <c r="C14">
+        <v>0</v>
+      </c>
+      <c r="D14" t="s">
+        <v>33</v>
+      </c>
+      <c r="E14" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>35</v>
+      </c>
+      <c r="B15" s="1">
+        <v>8.7699999999999996E-4</v>
+      </c>
+      <c r="C15" s="1">
+        <v>8.52E-4</v>
+      </c>
+      <c r="D15" t="s">
+        <v>36</v>
+      </c>
+      <c r="E15" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>38</v>
+      </c>
+      <c r="B16" s="1">
+        <v>2.55E-5</v>
+      </c>
+      <c r="C16" s="1">
+        <v>2.55E-5</v>
+      </c>
+      <c r="D16" t="s">
+        <v>39</v>
+      </c>
+      <c r="E16" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>41</v>
+      </c>
+      <c r="B17" s="1">
+        <v>6.3299999999999994E-5</v>
+      </c>
+      <c r="C17" s="1">
+        <v>6.3299999999999994E-5</v>
+      </c>
+      <c r="D17" t="s">
+        <v>42</v>
+      </c>
+      <c r="E17" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>50</v>
+      </c>
+      <c r="B18" s="1">
+        <v>5.4799999999999997E-5</v>
+      </c>
+      <c r="C18" s="1">
+        <v>5.4799999999999997E-5</v>
+      </c>
+      <c r="D18" t="s">
+        <v>51</v>
+      </c>
+      <c r="E18" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>44</v>
+      </c>
+      <c r="B19" s="1">
+        <v>3.6600000000000002E-5</v>
+      </c>
+      <c r="C19" s="1">
+        <v>1.9700000000000001E-5</v>
+      </c>
+      <c r="D19" t="s">
+        <v>45</v>
+      </c>
+      <c r="E19" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>47</v>
+      </c>
+      <c r="B20" s="1">
+        <v>1.6900000000000001E-5</v>
+      </c>
+      <c r="C20" s="1">
+        <v>1.6900000000000001E-5</v>
+      </c>
+      <c r="D20" t="s">
+        <v>48</v>
+      </c>
+      <c r="E20" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>53</v>
+      </c>
+      <c r="B21" s="1">
+        <v>3.4199999999999998E-5</v>
+      </c>
+      <c r="C21" s="1">
+        <v>3.4199999999999998E-5</v>
+      </c>
+      <c r="D21" t="s">
+        <v>54</v>
+      </c>
+      <c r="E21" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>59</v>
+      </c>
+      <c r="B22" s="1">
+        <v>8.8799999999999997E-6</v>
+      </c>
+      <c r="C22" s="1">
+        <v>8.8799999999999997E-6</v>
+      </c>
+      <c r="D22" t="s">
+        <v>60</v>
+      </c>
+      <c r="E22" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>56</v>
+      </c>
+      <c r="B23" s="1">
+        <v>2.4200000000000001E-6</v>
+      </c>
+      <c r="C23" s="1">
+        <v>2.4200000000000001E-6</v>
+      </c>
+      <c r="D23" t="s">
+        <v>57</v>
+      </c>
+      <c r="E23" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>61</v>
+      </c>
+      <c r="B24">
+        <v>1E-3</v>
+      </c>
+      <c r="C24" s="1">
+        <v>7.17E-6</v>
+      </c>
+      <c r="D24" t="s">
+        <v>62</v>
+      </c>
+      <c r="E24" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B25">
+        <v>1E-3</v>
+      </c>
+      <c r="C25">
+        <v>1E-3</v>
+      </c>
+      <c r="D25" t="s">
+        <v>65</v>
+      </c>
+      <c r="E25" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>67</v>
+      </c>
+      <c r="B26" s="1">
+        <v>5.8199999999999998E-5</v>
+      </c>
+      <c r="C26" s="1">
+        <v>5.8199999999999998E-5</v>
+      </c>
+      <c r="D26" t="s">
+        <v>68</v>
+      </c>
+      <c r="E26" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>70</v>
+      </c>
+      <c r="B27" s="1">
+        <v>4.6300000000000001E-5</v>
+      </c>
+      <c r="C27" s="1">
+        <v>4.6300000000000001E-5</v>
+      </c>
+      <c r="D27" t="s">
+        <v>71</v>
+      </c>
+      <c r="E27" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>73</v>
+      </c>
+      <c r="B28" s="1">
+        <v>1.01E-5</v>
+      </c>
+      <c r="C28" s="1">
+        <v>1.01E-5</v>
+      </c>
+      <c r="D28" t="s">
+        <v>74</v>
+      </c>
+      <c r="E28" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>76</v>
+      </c>
+      <c r="B29" s="1">
+        <v>4.8099999999999997E-6</v>
+      </c>
+      <c r="C29" s="1">
+        <v>4.8099999999999997E-6</v>
+      </c>
+      <c r="D29" t="s">
+        <v>77</v>
+      </c>
+      <c r="E29" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>79</v>
+      </c>
+      <c r="B30" s="1">
+        <v>4.3000000000000003E-6</v>
+      </c>
+      <c r="C30" s="1">
+        <v>4.3000000000000003E-6</v>
+      </c>
+      <c r="D30" t="s">
+        <v>80</v>
+      </c>
+      <c r="E30" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>87</v>
+      </c>
+      <c r="B31" s="1">
+        <v>9.1600000000000004E-4</v>
+      </c>
+      <c r="C31" s="1">
+        <v>9.7299999999999993E-5</v>
+      </c>
+      <c r="D31" t="s">
+        <v>88</v>
+      </c>
+      <c r="E31" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>90</v>
+      </c>
+      <c r="B32" s="1">
+        <v>7.6800000000000002E-4</v>
+      </c>
+      <c r="C32" s="1">
+        <v>7.6800000000000002E-4</v>
+      </c>
+      <c r="D32" t="s">
+        <v>91</v>
+      </c>
+      <c r="E32" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>93</v>
+      </c>
+      <c r="B33" s="1">
+        <v>4.9700000000000002E-5</v>
+      </c>
+      <c r="C33" s="1">
+        <v>4.9700000000000002E-5</v>
+      </c>
+      <c r="D33" t="s">
+        <v>94</v>
+      </c>
+      <c r="E33" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>82</v>
+      </c>
+      <c r="B34" s="1">
+        <v>8.6399999999999997E-4</v>
+      </c>
+      <c r="C34" s="1">
+        <v>8.6399999999999997E-4</v>
+      </c>
+      <c r="D34" t="s">
+        <v>83</v>
+      </c>
+      <c r="E34" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>96</v>
+      </c>
+      <c r="B35" s="1">
+        <v>6.3100000000000005E-4</v>
+      </c>
+      <c r="C35" s="1">
+        <v>6.3100000000000005E-4</v>
+      </c>
+      <c r="D35" t="s">
+        <v>97</v>
+      </c>
+      <c r="E35" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>85</v>
+      </c>
+      <c r="B36" s="1">
+        <v>3.3399999999999999E-4</v>
+      </c>
+      <c r="C36" s="1">
+        <v>3.3399999999999999E-4</v>
+      </c>
+      <c r="D36" t="s">
+        <v>86</v>
+      </c>
+      <c r="E36" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>98</v>
+      </c>
+      <c r="B37" s="1">
+        <v>1.11E-4</v>
+      </c>
+      <c r="C37" s="1">
+        <v>1.11E-4</v>
+      </c>
+      <c r="D37" t="s">
+        <v>99</v>
+      </c>
+      <c r="E37" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>115</v>
+      </c>
+      <c r="B38" s="1">
+        <v>1.06E-4</v>
+      </c>
+      <c r="C38" s="1">
+        <v>1.06E-4</v>
+      </c>
+      <c r="D38" t="s">
+        <v>116</v>
+      </c>
+      <c r="E38" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>128</v>
+      </c>
+      <c r="B39" s="1">
+        <v>8.7700000000000004E-5</v>
+      </c>
+      <c r="C39" s="1">
+        <v>8.7700000000000004E-5</v>
+      </c>
+      <c r="D39" t="s">
+        <v>129</v>
+      </c>
+      <c r="E39" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>117</v>
+      </c>
+      <c r="B40" s="1">
+        <v>8.7499999999999999E-5</v>
+      </c>
+      <c r="C40" s="1">
+        <v>8.7499999999999999E-5</v>
+      </c>
+      <c r="D40" t="s">
+        <v>118</v>
+      </c>
+      <c r="E40" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>101</v>
+      </c>
+      <c r="B41" s="1">
+        <v>3.5800000000000003E-5</v>
+      </c>
+      <c r="C41" s="1">
+        <v>3.5800000000000003E-5</v>
+      </c>
+      <c r="D41" t="s">
+        <v>102</v>
+      </c>
+      <c r="E41" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>105</v>
+      </c>
+      <c r="B42" s="1">
+        <v>3.4499999999999998E-5</v>
+      </c>
+      <c r="C42" s="1">
+        <v>3.4499999999999998E-5</v>
+      </c>
+      <c r="D42" t="s">
+        <v>106</v>
+      </c>
+      <c r="E42" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>109</v>
+      </c>
+      <c r="B43" s="1">
+        <v>3.1199999999999999E-5</v>
+      </c>
+      <c r="C43" s="1">
+        <v>3.1199999999999999E-5</v>
+      </c>
+      <c r="D43" t="s">
+        <v>110</v>
+      </c>
+      <c r="E43" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>121</v>
+      </c>
+      <c r="B44" s="1">
+        <v>2.5999999999999998E-5</v>
+      </c>
+      <c r="C44" s="1">
+        <v>2.5999999999999998E-5</v>
+      </c>
+      <c r="D44" t="s">
+        <v>122</v>
+      </c>
+      <c r="E44" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>103</v>
+      </c>
+      <c r="B45" s="1">
+        <v>2.23E-5</v>
+      </c>
+      <c r="C45" s="1">
+        <v>2.23E-5</v>
+      </c>
+      <c r="D45" t="s">
+        <v>104</v>
+      </c>
+      <c r="E45" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>107</v>
+      </c>
+      <c r="B46" s="1">
+        <v>1.9400000000000001E-5</v>
+      </c>
+      <c r="C46" s="1">
+        <v>1.9400000000000001E-5</v>
+      </c>
+      <c r="D46" t="s">
+        <v>108</v>
+      </c>
+      <c r="E46" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>111</v>
+      </c>
+      <c r="B47" s="1">
+        <v>1.7399999999999999E-5</v>
+      </c>
+      <c r="C47" s="1">
+        <v>1.7399999999999999E-5</v>
+      </c>
+      <c r="D47" t="s">
+        <v>112</v>
+      </c>
+      <c r="E47" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>113</v>
+      </c>
+      <c r="B48" s="1">
+        <v>1.7200000000000001E-5</v>
+      </c>
+      <c r="C48" s="1">
+        <v>1.7200000000000001E-5</v>
+      </c>
+      <c r="D48" t="s">
+        <v>114</v>
+      </c>
+      <c r="E48" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>130</v>
+      </c>
+      <c r="B49" s="1">
+        <v>1.5500000000000001E-5</v>
+      </c>
+      <c r="C49" s="1">
+        <v>1.5500000000000001E-5</v>
+      </c>
+      <c r="D49" t="s">
+        <v>131</v>
+      </c>
+      <c r="E49" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>132</v>
+      </c>
+      <c r="B50" s="1">
+        <v>1.19E-5</v>
+      </c>
+      <c r="C50" s="1">
+        <v>1.19E-5</v>
+      </c>
+      <c r="D50" t="s">
+        <v>133</v>
+      </c>
+      <c r="E50" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>119</v>
+      </c>
+      <c r="B51" s="1">
+        <v>9.4099999999999997E-6</v>
+      </c>
+      <c r="C51" s="1">
+        <v>9.4099999999999997E-6</v>
+      </c>
+      <c r="D51" t="s">
+        <v>120</v>
+      </c>
+      <c r="E51" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>126</v>
+      </c>
+      <c r="B52" s="1">
+        <v>9.1800000000000002E-6</v>
+      </c>
+      <c r="C52" s="1">
+        <v>9.1800000000000002E-6</v>
+      </c>
+      <c r="D52" t="s">
+        <v>127</v>
+      </c>
+      <c r="E52" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>123</v>
+      </c>
+      <c r="B53" s="1">
+        <v>4.0500000000000002E-6</v>
+      </c>
+      <c r="C53" s="1">
+        <v>4.0500000000000002E-6</v>
+      </c>
+      <c r="D53" t="s">
+        <v>124</v>
+      </c>
+      <c r="E53" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>134</v>
+      </c>
+      <c r="B54" s="1">
+        <v>2.7199999999999998E-6</v>
+      </c>
+      <c r="C54" s="1">
+        <v>2.7199999999999998E-6</v>
+      </c>
+      <c r="D54" t="s">
+        <v>135</v>
+      </c>
+      <c r="E54" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>136</v>
+      </c>
+      <c r="B55" s="1">
+        <v>2.5900000000000002E-6</v>
+      </c>
+      <c r="C55" s="1">
+        <v>2.5900000000000002E-6</v>
+      </c>
+      <c r="D55" t="s">
+        <v>137</v>
+      </c>
+      <c r="E55" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>138</v>
+      </c>
+      <c r="B56" s="1">
+        <v>1.9199999999999998E-6</v>
+      </c>
+      <c r="C56" s="1">
+        <v>1.9199999999999998E-6</v>
+      </c>
+      <c r="D56" t="s">
+        <v>139</v>
+      </c>
+      <c r="E56" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>140</v>
+      </c>
+      <c r="B57" s="1">
+        <v>8.8700000000000004E-7</v>
+      </c>
+      <c r="C57" s="1">
+        <v>8.8700000000000004E-7</v>
+      </c>
+      <c r="D57" t="s">
+        <v>141</v>
+      </c>
+      <c r="E57" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>142</v>
+      </c>
+      <c r="B58" s="1">
+        <v>5.7800000000000001E-7</v>
+      </c>
+      <c r="C58" s="1">
+        <v>5.7800000000000001E-7</v>
+      </c>
+      <c r="D58" t="s">
+        <v>143</v>
+      </c>
+      <c r="E58" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>146</v>
+      </c>
+      <c r="B59" s="1">
+        <v>5.2600000000000002E-7</v>
+      </c>
+      <c r="C59" s="1">
+        <v>5.2600000000000002E-7</v>
+      </c>
+      <c r="D59" t="s">
+        <v>147</v>
+      </c>
+      <c r="E59" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>148</v>
+      </c>
+      <c r="B60" s="1">
+        <v>5.2600000000000002E-7</v>
+      </c>
+      <c r="C60" s="1">
+        <v>5.2600000000000002E-7</v>
+      </c>
+      <c r="D60" t="s">
+        <v>149</v>
+      </c>
+      <c r="E60" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>150</v>
+      </c>
+      <c r="B61" s="1">
+        <v>5.2600000000000002E-7</v>
+      </c>
+      <c r="C61" s="1">
+        <v>5.2600000000000002E-7</v>
+      </c>
+      <c r="D61" t="s">
+        <v>151</v>
+      </c>
+      <c r="E61" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>144</v>
+      </c>
+      <c r="B62" s="1">
+        <v>4.6899999999999998E-7</v>
+      </c>
+      <c r="C62" s="1">
+        <v>4.6899999999999998E-7</v>
+      </c>
+      <c r="D62" t="s">
+        <v>145</v>
+      </c>
+      <c r="E62" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>152</v>
+      </c>
+      <c r="B63" s="1">
+        <v>2.9999999999999999E-7</v>
+      </c>
+      <c r="C63" s="1">
+        <v>2.9999999999999999E-7</v>
+      </c>
+      <c r="D63" t="s">
+        <v>153</v>
+      </c>
+      <c r="E63" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>154</v>
+      </c>
+      <c r="B64" s="1">
+        <v>2.96E-7</v>
+      </c>
+      <c r="C64" s="1">
+        <v>2.96E-7</v>
+      </c>
+      <c r="D64" t="s">
+        <v>155</v>
+      </c>
+      <c r="E64" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>156</v>
+      </c>
+      <c r="B65" s="1">
+        <v>5.7200000000000003E-4</v>
+      </c>
+      <c r="C65">
+        <v>0</v>
+      </c>
+      <c r="D65" t="s">
+        <v>157</v>
+      </c>
+      <c r="E65" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>159</v>
+      </c>
+      <c r="B66" s="1">
+        <v>5.7200000000000003E-4</v>
+      </c>
+      <c r="C66">
+        <v>0</v>
+      </c>
+      <c r="D66" t="s">
+        <v>160</v>
+      </c>
+      <c r="E66" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>32</v>
+      </c>
+      <c r="B67" s="1">
+        <v>5.7200000000000003E-4</v>
+      </c>
+      <c r="C67">
+        <v>0</v>
+      </c>
+      <c r="D67" t="s">
+        <v>161</v>
+      </c>
+      <c r="E67" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>35</v>
+      </c>
+      <c r="B68" s="1">
+        <v>5.7200000000000003E-4</v>
+      </c>
+      <c r="C68" s="1">
+        <v>5.7200000000000003E-4</v>
+      </c>
+      <c r="D68" t="s">
+        <v>163</v>
+      </c>
+      <c r="E68" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>165</v>
+      </c>
+      <c r="B69" s="1">
+        <v>3.8700000000000001E-7</v>
+      </c>
+      <c r="C69" s="1">
+        <v>3.8700000000000001E-7</v>
+      </c>
+      <c r="D69" t="s">
+        <v>166</v>
+      </c>
+      <c r="E69" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>38</v>
+      </c>
+      <c r="B70" s="1">
+        <v>5.1399999999999998E-10</v>
+      </c>
+      <c r="C70" s="1">
+        <v>5.1399999999999998E-10</v>
+      </c>
+      <c r="D70" t="s">
+        <v>168</v>
+      </c>
+      <c r="E70" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>169</v>
+      </c>
+      <c r="B71" s="1">
+        <v>1.15E-4</v>
+      </c>
+      <c r="C71" s="1">
+        <v>1.15E-4</v>
+      </c>
+      <c r="D71" t="s">
+        <v>170</v>
+      </c>
+      <c r="E71" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>172</v>
+      </c>
+      <c r="B72" s="1">
+        <v>2.0699999999999998E-5</v>
+      </c>
+      <c r="C72" s="1">
+        <v>2.0699999999999998E-5</v>
+      </c>
+      <c r="D72" t="s">
+        <v>173</v>
+      </c>
+      <c r="E72" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>175</v>
+      </c>
+      <c r="B73" s="1">
+        <v>5.5700000000000002E-7</v>
+      </c>
+      <c r="C73" s="1">
+        <v>5.5700000000000002E-7</v>
+      </c>
+      <c r="D73" t="s">
+        <v>176</v>
+      </c>
+      <c r="E73" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>178</v>
+      </c>
+      <c r="B74">
+        <v>0</v>
+      </c>
+      <c r="C74">
+        <v>0</v>
+      </c>
+      <c r="D74" t="s">
+        <v>179</v>
+      </c>
+      <c r="E74" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>181</v>
+      </c>
+      <c r="B75">
+        <v>0</v>
+      </c>
+      <c r="C75">
+        <v>0</v>
+      </c>
+      <c r="D75" t="s">
+        <v>182</v>
+      </c>
+      <c r="E75" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>184</v>
+      </c>
+      <c r="B76">
+        <v>0</v>
+      </c>
+      <c r="C76">
+        <v>0</v>
+      </c>
+      <c r="D76" t="s">
+        <v>185</v>
+      </c>
+      <c r="E76" t="s">
+        <v>186</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAE15965-3211-4FBB-8692-E47112645D65}">
+  <dimension ref="A1:E76"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="28.7109375" customWidth="1"/>
+    <col min="2" max="2" width="39.5703125" customWidth="1"/>
+    <col min="3" max="3" width="41.42578125" customWidth="1"/>
+    <col min="4" max="4" width="96.7109375" customWidth="1"/>
+    <col min="5" max="5" width="57.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>0.33400000000000002</v>
+      </c>
+      <c r="C2">
+        <v>0.27200000000000002</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>6.2E-2</v>
+      </c>
+      <c r="C3">
+        <v>1.0999999999999999E-2</v>
+      </c>
+      <c r="E3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>4.5999999999999999E-2</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5">
+        <v>4.5999999999999999E-2</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>4.5999999999999999E-2</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7">
+        <v>4.5999999999999999E-2</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8">
+        <v>4.5999999999999999E-2</v>
+      </c>
+      <c r="C8">
+        <v>4.5999999999999999E-2</v>
+      </c>
+      <c r="D8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="C9" s="1">
+        <v>4.8299999999999998E-4</v>
+      </c>
+      <c r="D9" t="s">
+        <v>18</v>
+      </c>
+      <c r="E9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" s="1">
+        <v>9.4300000000000004E-4</v>
+      </c>
+      <c r="C10" s="1">
+        <v>2.1999999999999999E-5</v>
+      </c>
+      <c r="D10" t="s">
+        <v>21</v>
+      </c>
+      <c r="E10" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" s="1">
+        <v>7.6199999999999998E-4</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="1">
+        <v>7.6199999999999998E-4</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13" s="1">
+        <v>7.6199999999999998E-4</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
+      </c>
+      <c r="D13" t="s">
+        <v>30</v>
+      </c>
+      <c r="E13" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" s="1">
+        <v>7.6199999999999998E-4</v>
+      </c>
+      <c r="C14">
+        <v>0</v>
+      </c>
+      <c r="D14" t="s">
+        <v>33</v>
+      </c>
+      <c r="E14" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>35</v>
+      </c>
+      <c r="B15" s="1">
+        <v>7.6199999999999998E-4</v>
+      </c>
+      <c r="C15" s="1">
+        <v>7.4399999999999998E-4</v>
+      </c>
+      <c r="D15" t="s">
+        <v>36</v>
+      </c>
+      <c r="E15" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>38</v>
+      </c>
+      <c r="B16" s="1">
+        <v>1.7799999999999999E-5</v>
+      </c>
+      <c r="C16" s="1">
+        <v>1.7799999999999999E-5</v>
+      </c>
+      <c r="D16" t="s">
+        <v>39</v>
+      </c>
+      <c r="E16" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>41</v>
+      </c>
+      <c r="B17" s="1">
+        <v>6.2799999999999995E-5</v>
+      </c>
+      <c r="C17" s="1">
+        <v>6.2799999999999995E-5</v>
+      </c>
+      <c r="D17" t="s">
+        <v>42</v>
+      </c>
+      <c r="E17" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>50</v>
+      </c>
+      <c r="B18" s="1">
+        <v>3.2499999999999997E-5</v>
+      </c>
+      <c r="C18" s="1">
+        <v>3.2499999999999997E-5</v>
+      </c>
+      <c r="D18" t="s">
+        <v>51</v>
+      </c>
+      <c r="E18" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>44</v>
+      </c>
+      <c r="B19" s="1">
+        <v>2.8200000000000001E-5</v>
+      </c>
+      <c r="C19" s="1">
+        <v>1.4800000000000001E-5</v>
+      </c>
+      <c r="D19" t="s">
+        <v>45</v>
+      </c>
+      <c r="E19" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>47</v>
+      </c>
+      <c r="B20" s="1">
+        <v>1.34E-5</v>
+      </c>
+      <c r="C20" s="1">
+        <v>1.34E-5</v>
+      </c>
+      <c r="D20" t="s">
+        <v>48</v>
+      </c>
+      <c r="E20" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>53</v>
+      </c>
+      <c r="B21" s="1">
+        <v>2.6100000000000001E-5</v>
+      </c>
+      <c r="C21" s="1">
+        <v>2.6100000000000001E-5</v>
+      </c>
+      <c r="D21" t="s">
+        <v>54</v>
+      </c>
+      <c r="E21" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>59</v>
+      </c>
+      <c r="B22" s="1">
+        <v>5.4500000000000003E-6</v>
+      </c>
+      <c r="C22" s="1">
+        <v>5.4500000000000003E-6</v>
+      </c>
+      <c r="D22" t="s">
+        <v>60</v>
+      </c>
+      <c r="E22" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>56</v>
+      </c>
+      <c r="B23" s="1">
+        <v>4.0899999999999998E-6</v>
+      </c>
+      <c r="C23" s="1">
+        <v>4.0899999999999998E-6</v>
+      </c>
+      <c r="D23" t="s">
+        <v>57</v>
+      </c>
+      <c r="E23" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>61</v>
+      </c>
+      <c r="B24" s="1">
+        <v>8.6799999999999996E-4</v>
+      </c>
+      <c r="C24" s="1">
+        <v>5.2599999999999996E-6</v>
+      </c>
+      <c r="D24" t="s">
+        <v>62</v>
+      </c>
+      <c r="E24" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B25" s="1">
+        <v>7.3899999999999997E-4</v>
+      </c>
+      <c r="C25" s="1">
+        <v>7.3899999999999997E-4</v>
+      </c>
+      <c r="D25" t="s">
+        <v>65</v>
+      </c>
+      <c r="E25" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>70</v>
+      </c>
+      <c r="B26" s="1">
+        <v>7.6500000000000003E-5</v>
+      </c>
+      <c r="C26" s="1">
+        <v>7.6500000000000003E-5</v>
+      </c>
+      <c r="D26" t="s">
+        <v>71</v>
+      </c>
+      <c r="E26" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>67</v>
+      </c>
+      <c r="B27" s="1">
+        <v>3.1900000000000003E-5</v>
+      </c>
+      <c r="C27" s="1">
+        <v>3.1900000000000003E-5</v>
+      </c>
+      <c r="D27" t="s">
+        <v>68</v>
+      </c>
+      <c r="E27" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>79</v>
+      </c>
+      <c r="B28" s="1">
+        <v>9.0000000000000002E-6</v>
+      </c>
+      <c r="C28" s="1">
+        <v>9.0000000000000002E-6</v>
+      </c>
+      <c r="D28" t="s">
+        <v>80</v>
+      </c>
+      <c r="E28" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>73</v>
+      </c>
+      <c r="B29" s="1">
+        <v>4.7199999999999997E-6</v>
+      </c>
+      <c r="C29" s="1">
+        <v>4.7199999999999997E-6</v>
+      </c>
+      <c r="D29" t="s">
+        <v>74</v>
+      </c>
+      <c r="E29" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>76</v>
+      </c>
+      <c r="B30" s="1">
+        <v>2.3800000000000001E-6</v>
+      </c>
+      <c r="C30" s="1">
+        <v>2.3800000000000001E-6</v>
+      </c>
+      <c r="D30" t="s">
+        <v>77</v>
+      </c>
+      <c r="E30" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>87</v>
+      </c>
+      <c r="B31" s="1">
+        <v>6.5700000000000003E-4</v>
+      </c>
+      <c r="C31" s="1">
+        <v>1.02E-4</v>
+      </c>
+      <c r="D31" t="s">
+        <v>88</v>
+      </c>
+      <c r="E31" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>90</v>
+      </c>
+      <c r="B32" s="1">
+        <v>5.1099999999999995E-4</v>
+      </c>
+      <c r="C32" s="1">
+        <v>5.1099999999999995E-4</v>
+      </c>
+      <c r="D32" t="s">
+        <v>91</v>
+      </c>
+      <c r="E32" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>93</v>
+      </c>
+      <c r="B33" s="1">
+        <v>4.3800000000000001E-5</v>
+      </c>
+      <c r="C33" s="1">
+        <v>4.3800000000000001E-5</v>
+      </c>
+      <c r="D33" t="s">
+        <v>94</v>
+      </c>
+      <c r="E33" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>82</v>
+      </c>
+      <c r="B34" s="1">
+        <v>3.9300000000000001E-4</v>
+      </c>
+      <c r="C34" s="1">
+        <v>3.9300000000000001E-4</v>
+      </c>
+      <c r="D34" t="s">
+        <v>83</v>
+      </c>
+      <c r="E34" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>96</v>
+      </c>
+      <c r="B35" s="1">
+        <v>3.8400000000000001E-4</v>
+      </c>
+      <c r="C35" s="1">
+        <v>3.8400000000000001E-4</v>
+      </c>
+      <c r="D35" t="s">
+        <v>97</v>
+      </c>
+      <c r="E35" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>85</v>
+      </c>
+      <c r="B36" s="1">
+        <v>2.0699999999999999E-4</v>
+      </c>
+      <c r="C36" s="1">
+        <v>2.0699999999999999E-4</v>
+      </c>
+      <c r="D36" t="s">
+        <v>86</v>
+      </c>
+      <c r="E36" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>98</v>
+      </c>
+      <c r="B37" s="1">
+        <v>1.92E-4</v>
+      </c>
+      <c r="C37" s="1">
+        <v>1.92E-4</v>
+      </c>
+      <c r="D37" t="s">
+        <v>99</v>
+      </c>
+      <c r="E37" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>115</v>
+      </c>
+      <c r="B38" s="1">
+        <v>8.5599999999999994E-5</v>
+      </c>
+      <c r="C38" s="1">
+        <v>8.5599999999999994E-5</v>
+      </c>
+      <c r="D38" t="s">
+        <v>116</v>
+      </c>
+      <c r="E38" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>117</v>
+      </c>
+      <c r="B39" s="1">
+        <v>7.8100000000000001E-5</v>
+      </c>
+      <c r="C39" s="1">
+        <v>7.8100000000000001E-5</v>
+      </c>
+      <c r="D39" t="s">
+        <v>118</v>
+      </c>
+      <c r="E39" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>101</v>
+      </c>
+      <c r="B40" s="1">
+        <v>4.2799999999999997E-5</v>
+      </c>
+      <c r="C40" s="1">
+        <v>4.2799999999999997E-5</v>
+      </c>
+      <c r="D40" t="s">
+        <v>102</v>
+      </c>
+      <c r="E40" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>105</v>
+      </c>
+      <c r="B41" s="1">
+        <v>3.9799999999999998E-5</v>
+      </c>
+      <c r="C41" s="1">
+        <v>3.9799999999999998E-5</v>
+      </c>
+      <c r="D41" t="s">
+        <v>106</v>
+      </c>
+      <c r="E41" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>103</v>
+      </c>
+      <c r="B42" s="1">
+        <v>3.96E-5</v>
+      </c>
+      <c r="C42" s="1">
+        <v>3.96E-5</v>
+      </c>
+      <c r="D42" t="s">
+        <v>104</v>
+      </c>
+      <c r="E42" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>111</v>
+      </c>
+      <c r="B43" s="1">
+        <v>3.1199999999999999E-5</v>
+      </c>
+      <c r="C43" s="1">
+        <v>3.1199999999999999E-5</v>
+      </c>
+      <c r="D43" t="s">
+        <v>112</v>
+      </c>
+      <c r="E43" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>113</v>
+      </c>
+      <c r="B44" s="1">
+        <v>2.9899999999999998E-5</v>
+      </c>
+      <c r="C44" s="1">
+        <v>2.9899999999999998E-5</v>
+      </c>
+      <c r="D44" t="s">
+        <v>114</v>
+      </c>
+      <c r="E44" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>148</v>
+      </c>
+      <c r="B45" s="1">
+        <v>2.9499999999999999E-5</v>
+      </c>
+      <c r="C45" s="1">
+        <v>2.9499999999999999E-5</v>
+      </c>
+      <c r="D45" t="s">
+        <v>149</v>
+      </c>
+      <c r="E45" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>150</v>
+      </c>
+      <c r="B46" s="1">
+        <v>2.55E-5</v>
+      </c>
+      <c r="C46" s="1">
+        <v>2.55E-5</v>
+      </c>
+      <c r="D46" t="s">
+        <v>151</v>
+      </c>
+      <c r="E46" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>109</v>
+      </c>
+      <c r="B47" s="1">
+        <v>2.4600000000000002E-5</v>
+      </c>
+      <c r="C47" s="1">
+        <v>2.4600000000000002E-5</v>
+      </c>
+      <c r="D47" t="s">
+        <v>110</v>
+      </c>
+      <c r="E47" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>107</v>
+      </c>
+      <c r="B48" s="1">
+        <v>2.4199999999999999E-5</v>
+      </c>
+      <c r="C48" s="1">
+        <v>2.4199999999999999E-5</v>
+      </c>
+      <c r="D48" t="s">
+        <v>108</v>
+      </c>
+      <c r="E48" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>126</v>
+      </c>
+      <c r="B49" s="1">
+        <v>2.34E-5</v>
+      </c>
+      <c r="C49" s="1">
+        <v>2.34E-5</v>
+      </c>
+      <c r="D49" t="s">
+        <v>127</v>
+      </c>
+      <c r="E49" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>121</v>
+      </c>
+      <c r="B50" s="1">
+        <v>2.0599999999999999E-5</v>
+      </c>
+      <c r="C50" s="1">
+        <v>2.0599999999999999E-5</v>
+      </c>
+      <c r="D50" t="s">
+        <v>122</v>
+      </c>
+      <c r="E50" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>119</v>
+      </c>
+      <c r="B51" s="1">
+        <v>1.52E-5</v>
+      </c>
+      <c r="C51" s="1">
+        <v>1.52E-5</v>
+      </c>
+      <c r="D51" t="s">
+        <v>120</v>
+      </c>
+      <c r="E51" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>128</v>
+      </c>
+      <c r="B52" s="1">
+        <v>1.27E-5</v>
+      </c>
+      <c r="C52" s="1">
+        <v>1.27E-5</v>
+      </c>
+      <c r="D52" t="s">
+        <v>129</v>
+      </c>
+      <c r="E52" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>132</v>
+      </c>
+      <c r="B53" s="1">
+        <v>1.2300000000000001E-5</v>
+      </c>
+      <c r="C53" s="1">
+        <v>1.2300000000000001E-5</v>
+      </c>
+      <c r="D53" t="s">
+        <v>133</v>
+      </c>
+      <c r="E53" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>130</v>
+      </c>
+      <c r="B54" s="1">
+        <v>1.1199999999999999E-5</v>
+      </c>
+      <c r="C54" s="1">
+        <v>1.1199999999999999E-5</v>
+      </c>
+      <c r="D54" t="s">
+        <v>131</v>
+      </c>
+      <c r="E54" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>154</v>
+      </c>
+      <c r="B55" s="1">
+        <v>9.2199999999999998E-6</v>
+      </c>
+      <c r="C55" s="1">
+        <v>9.2199999999999998E-6</v>
+      </c>
+      <c r="D55" t="s">
+        <v>155</v>
+      </c>
+      <c r="E55" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>134</v>
+      </c>
+      <c r="B56" s="1">
+        <v>6.3400000000000003E-6</v>
+      </c>
+      <c r="C56" s="1">
+        <v>6.3400000000000003E-6</v>
+      </c>
+      <c r="D56" t="s">
+        <v>135</v>
+      </c>
+      <c r="E56" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>136</v>
+      </c>
+      <c r="B57" s="1">
+        <v>5.8900000000000004E-6</v>
+      </c>
+      <c r="C57" s="1">
+        <v>5.8900000000000004E-6</v>
+      </c>
+      <c r="D57" t="s">
+        <v>137</v>
+      </c>
+      <c r="E57" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>138</v>
+      </c>
+      <c r="B58" s="1">
+        <v>4.2400000000000001E-6</v>
+      </c>
+      <c r="C58" s="1">
+        <v>4.2400000000000001E-6</v>
+      </c>
+      <c r="D58" t="s">
+        <v>139</v>
+      </c>
+      <c r="E58" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>123</v>
+      </c>
+      <c r="B59" s="1">
+        <v>3.4999999999999999E-6</v>
+      </c>
+      <c r="C59" s="1">
+        <v>3.4999999999999999E-6</v>
+      </c>
+      <c r="D59" t="s">
+        <v>124</v>
+      </c>
+      <c r="E59" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>140</v>
+      </c>
+      <c r="B60" s="1">
+        <v>1.2899999999999999E-6</v>
+      </c>
+      <c r="C60" s="1">
+        <v>1.2899999999999999E-6</v>
+      </c>
+      <c r="D60" t="s">
+        <v>141</v>
+      </c>
+      <c r="E60" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>142</v>
+      </c>
+      <c r="B61" s="1">
+        <v>7.7100000000000001E-7</v>
+      </c>
+      <c r="C61" s="1">
+        <v>7.7100000000000001E-7</v>
+      </c>
+      <c r="D61" t="s">
+        <v>143</v>
+      </c>
+      <c r="E61" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>146</v>
+      </c>
+      <c r="B62" s="1">
+        <v>5.2600000000000002E-7</v>
+      </c>
+      <c r="C62" s="1">
+        <v>5.2600000000000002E-7</v>
+      </c>
+      <c r="D62" t="s">
+        <v>147</v>
+      </c>
+      <c r="E62" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>144</v>
+      </c>
+      <c r="B63" s="1">
+        <v>4.3500000000000002E-7</v>
+      </c>
+      <c r="C63" s="1">
+        <v>4.3500000000000002E-7</v>
+      </c>
+      <c r="D63" t="s">
+        <v>145</v>
+      </c>
+      <c r="E63" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>152</v>
+      </c>
+      <c r="B64" s="1">
+        <v>3.2599999999999998E-7</v>
+      </c>
+      <c r="C64" s="1">
+        <v>3.2599999999999998E-7</v>
+      </c>
+      <c r="D64" t="s">
+        <v>153</v>
+      </c>
+      <c r="E64" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>156</v>
+      </c>
+      <c r="B65" s="1">
+        <v>7.0699999999999995E-4</v>
+      </c>
+      <c r="C65">
+        <v>0</v>
+      </c>
+      <c r="D65" t="s">
+        <v>157</v>
+      </c>
+      <c r="E65" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>159</v>
+      </c>
+      <c r="B66" s="1">
+        <v>7.0699999999999995E-4</v>
+      </c>
+      <c r="C66">
+        <v>0</v>
+      </c>
+      <c r="D66" t="s">
+        <v>160</v>
+      </c>
+      <c r="E66" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>32</v>
+      </c>
+      <c r="B67" s="1">
+        <v>7.0699999999999995E-4</v>
+      </c>
+      <c r="C67">
+        <v>0</v>
+      </c>
+      <c r="D67" t="s">
+        <v>161</v>
+      </c>
+      <c r="E67" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>35</v>
+      </c>
+      <c r="B68" s="1">
+        <v>7.0699999999999995E-4</v>
+      </c>
+      <c r="C68" s="1">
+        <v>7.0200000000000004E-4</v>
+      </c>
+      <c r="D68" t="s">
+        <v>163</v>
+      </c>
+      <c r="E68" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>38</v>
+      </c>
+      <c r="B69" s="1">
+        <v>4.6199999999999998E-6</v>
+      </c>
+      <c r="C69" s="1">
+        <v>4.6199999999999998E-6</v>
+      </c>
+      <c r="D69" t="s">
+        <v>168</v>
+      </c>
+      <c r="E69" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>165</v>
+      </c>
+      <c r="B70" s="1">
+        <v>1.37E-7</v>
+      </c>
+      <c r="C70" s="1">
+        <v>1.37E-7</v>
+      </c>
+      <c r="D70" t="s">
+        <v>166</v>
+      </c>
+      <c r="E70" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>169</v>
+      </c>
+      <c r="B71" s="1">
+        <v>1.37E-4</v>
+      </c>
+      <c r="C71" s="1">
+        <v>1.37E-4</v>
+      </c>
+      <c r="D71" t="s">
+        <v>170</v>
+      </c>
+      <c r="E71" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>172</v>
+      </c>
+      <c r="B72" s="1">
+        <v>2.62E-5</v>
+      </c>
+      <c r="C72" s="1">
+        <v>2.62E-5</v>
+      </c>
+      <c r="D72" t="s">
+        <v>173</v>
+      </c>
+      <c r="E72" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>175</v>
+      </c>
+      <c r="B73" s="1">
+        <v>5.5700000000000002E-7</v>
+      </c>
+      <c r="C73" s="1">
+        <v>5.5700000000000002E-7</v>
+      </c>
+      <c r="D73" t="s">
+        <v>176</v>
+      </c>
+      <c r="E73" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>178</v>
+      </c>
+      <c r="B74">
+        <v>0</v>
+      </c>
+      <c r="C74">
+        <v>0</v>
+      </c>
+      <c r="D74" t="s">
+        <v>179</v>
+      </c>
+      <c r="E74" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>181</v>
+      </c>
+      <c r="B75">
+        <v>0</v>
+      </c>
+      <c r="C75">
+        <v>0</v>
+      </c>
+      <c r="D75" t="s">
+        <v>182</v>
+      </c>
+      <c r="E75" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>184</v>
+      </c>
+      <c r="B76">
+        <v>0</v>
+      </c>
+      <c r="C76">
+        <v>0</v>
+      </c>
+      <c r="D76" t="s">
+        <v>185</v>
+      </c>
+      <c r="E76" t="s">
+        <v>186</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>